<commit_message>
[auto-snapshot] 2026-04-27 08:00 | onda-hompage | 145 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강북_PT.xlsx
+++ b/naver-place-crawler/results_health/강북_PT.xlsx
@@ -432,7 +432,7 @@
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="35" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
     <col width="10" customWidth="1" min="14" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
@@ -646,7 +646,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/97_cosat</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -690,24 +690,20 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wa2rxwt</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
           <t>X</t>
@@ -744,7 +740,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -778,7 +774,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/dwgym1</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -788,24 +784,20 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/w4e814</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
           <t>X</t>
@@ -842,7 +834,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -876,7 +868,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://www.instagram.com/lifebuildingpt/</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -886,7 +878,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -936,7 +928,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -970,7 +962,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>https://blog.naver.com/ready4gymsuyu</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -980,24 +972,20 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>O</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>O</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>https://talk.naver.com/ct/wcs9wn</t>
-        </is>
-      </c>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
           <t>X</t>
@@ -1009,13 +997,13 @@
         </is>
       </c>
       <c r="P6" t="n">
-        <v>1086</v>
+        <v>1085</v>
       </c>
       <c r="Q6" t="n">
         <v>870</v>
       </c>
       <c r="R6" t="n">
-        <v>1956</v>
+        <v>1955</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>
@@ -1034,7 +1022,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>
@@ -1128,7 +1116,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-27</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[auto-snapshot] 2026-04-27 12:00 | onda-hompage | 99 files
</commit_message>
<xml_diff>
--- a/naver-place-crawler/results_health/강북_PT.xlsx
+++ b/naver-place-crawler/results_health/강북_PT.xlsx
@@ -1000,10 +1000,10 @@
         <v>1085</v>
       </c>
       <c r="Q6" t="n">
-        <v>870</v>
+        <v>871</v>
       </c>
       <c r="R6" t="n">
-        <v>1955</v>
+        <v>1956</v>
       </c>
       <c r="S6" t="inlineStr">
         <is>

</xml_diff>